<commit_message>
feat: tabtools 2.4.0 regtab helpers; datamap 1.9.2 help links
tabtools 2.4.0 adds new regtab helper programs, including
_regtab_activeb.ado, _regtab_addcol.ado, _regtab_addrow.ado,
_regtab_cellnote.ado, _regtab_cmdopts.ado, _regtab_estats.ado,
_regtab_flatten.ado, _regtab_fvbase.ado, _regtab_methods.ado, and
_regtab_mstats.ado. It also changes _desctab_collect.ado and updates
tabtools/README.md. Separately, datamap 1.9.2 adds a Package commands
section at the top of datamap.sthlp that links to the help files for
datadict, datacheck, dataqa, and datamvp; the datamap .ado version
headers, datamap.pkg, and README were synced to 1.9.2 (2026/10/05)
without changing their logic. The root README.md version badges were
updated for both packages.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_comptab.xlsx
+++ b/tabtools/demo/demo_comptab.xlsx
@@ -11,13 +11,15 @@
     <sheet name="Composite" sheetId="3" r:id="rId5"/>
     <sheet name="Composite Compact" sheetId="4" r:id="rId6"/>
     <sheet name="Composite Names" sheetId="5" r:id="rId7"/>
+    <sheet name="Composite Formatted" sheetId="6" r:id="rId8"/>
+    <sheet name="Composite Flat" sheetId="7" r:id="rId9"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="231" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="286" uniqueCount="77">
   <si>
     <t>Cox Model -- Binary Treatment</t>
   </si>
@@ -55,13 +57,13 @@
     <t>1.00</t>
   </si>
   <si>
-    <t>1.01</t>
-  </si>
-  <si>
-    <t>1.53</t>
-  </si>
-  <si>
-    <t>1.50</t>
+    <t>1.02</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
+    <t>1.48</t>
   </si>
   <si>
     <t>1.69</t>
@@ -70,7 +72,7 @@
     <t>95% CI</t>
   </si>
   <si>
-    <t>(0.98, 1.10)</t>
+    <t>(0.97, 1.11)</t>
   </si>
   <si>
     <t>(1.00, 1.00)</t>
@@ -79,25 +81,25 @@
     <t>(0.96, 1.07)</t>
   </si>
   <si>
-    <t>(1.45, 1.62)</t>
-  </si>
-  <si>
-    <t>(1.42, 1.59)</t>
-  </si>
-  <si>
-    <t>(1.59, 1.80)</t>
+    <t>(1.42, 1.60)</t>
+  </si>
+  <si>
+    <t>(1.39, 1.57)</t>
+  </si>
+  <si>
+    <t>(1.60, 1.80)</t>
   </si>
   <si>
     <t>p-value</t>
   </si>
   <si>
-    <t>0.18</t>
-  </si>
-  <si>
-    <t>0.055</t>
-  </si>
-  <si>
-    <t>0.63</t>
+    <t>0.23</t>
+  </si>
+  <si>
+    <t>0.11</t>
+  </si>
+  <si>
+    <t>0.56</t>
   </si>
   <si>
     <t>&lt;0.001</t>
@@ -121,19 +123,19 @@
     <t>Reference</t>
   </si>
   <si>
-    <t>1.08</t>
+    <t>1.07</t>
   </si>
   <si>
     <t>1.05</t>
   </si>
   <si>
-    <t>1.02</t>
-  </si>
-  <si>
-    <t>1.58</t>
-  </si>
-  <si>
-    <t>1.54</t>
+    <t>1.03</t>
+  </si>
+  <si>
+    <t>1.55</t>
+  </si>
+  <si>
+    <t>1.52</t>
   </si>
   <si>
     <t>(1.00, 1.15)</t>
@@ -145,25 +147,28 @@
     <t>(0.97, 1.08)</t>
   </si>
   <si>
-    <t>(0.99, 1.10)</t>
-  </si>
-  <si>
-    <t>(1.50, 1.67)</t>
-  </si>
-  <si>
-    <t>(1.46, 1.63)</t>
-  </si>
-  <si>
-    <t>0.038</t>
-  </si>
-  <si>
-    <t>0.027</t>
-  </si>
-  <si>
-    <t>0.43</t>
-  </si>
-  <si>
-    <t>0.12</t>
+    <t>(0.98, 1.12)</t>
+  </si>
+  <si>
+    <t>(1.46, 1.65)</t>
+  </si>
+  <si>
+    <t>(1.43, 1.61)</t>
+  </si>
+  <si>
+    <t>0.042</t>
+  </si>
+  <si>
+    <t>0.19</t>
+  </si>
+  <si>
+    <t>0.064</t>
+  </si>
+  <si>
+    <t>0.37</t>
+  </si>
+  <si>
+    <t>0.21</t>
   </si>
   <si>
     <t>Table S1. Exposure Effects on Cardiovascular Events</t>
@@ -181,19 +186,19 @@
     <t>HR 95% CI</t>
   </si>
   <si>
-    <t>1.04 (0.98, 1.10)</t>
-  </si>
-  <si>
-    <t>1.53 (1.45, 1.62)</t>
-  </si>
-  <si>
-    <t>1.50 (1.42, 1.59)</t>
-  </si>
-  <si>
-    <t>1.69 (1.59, 1.80)</t>
-  </si>
-  <si>
-    <t>1.08 (1.00, 1.15)</t>
+    <t>1.04 (0.97, 1.11)</t>
+  </si>
+  <si>
+    <t>1.51 (1.42, 1.60)</t>
+  </si>
+  <si>
+    <t>1.48 (1.39, 1.57)</t>
+  </si>
+  <si>
+    <t>1.69 (1.60, 1.80)</t>
+  </si>
+  <si>
+    <t>1.07 (1.00, 1.15)</t>
   </si>
   <si>
     <t>1.05 (0.98, 1.13)</t>
@@ -206,6 +211,45 @@
   </si>
   <si>
     <t>Rows selected by label pattern using rownames() option.</t>
+  </si>
+  <si>
+    <t>Table S3. Selected Hazard Ratios (Three Decimals)</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>1.044</t>
+  </si>
+  <si>
+    <t>1.555</t>
+  </si>
+  <si>
+    <t>1.520</t>
+  </si>
+  <si>
+    <t>(0.976 to 1.117)</t>
+  </si>
+  <si>
+    <t>(1.464 to 1.651)</t>
+  </si>
+  <si>
+    <t>(1.432 to 1.614)</t>
+  </si>
+  <si>
+    <t>Table S3 flat frame written by puttab</t>
+  </si>
+  <si>
+    <t>rowlabel</t>
+  </si>
+  <si>
+    <t>Model, HR</t>
+  </si>
+  <si>
+    <t>Model, 95% CI</t>
+  </si>
+  <si>
+    <t>Model, p-value</t>
   </si>
 </sst>
 </file>
@@ -288,7 +332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -388,11 +432,18 @@
       <bottom style="medium"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -512,59 +563,47 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="bottom" wrapText="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="bottom" wrapText="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="general" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -877,7 +916,7 @@
         <v>40</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -894,7 +933,7 @@
         <v>18</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9">
@@ -911,7 +950,7 @@
         <v>41</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
@@ -922,13 +961,13 @@
         <v>2</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>42</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
@@ -988,7 +1027,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>1</v>
@@ -1119,7 +1158,7 @@
         <v>40</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1144,7 +1183,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="40" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B1" s="39" t="s">
         <v>1</v>
@@ -1178,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D3" s="36" t="s">
         <v>23</v>
@@ -1189,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C4" s="34" t="s">
         <v>1</v>
@@ -1206,7 +1245,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="29" t="s">
         <v>24</v>
@@ -1220,7 +1259,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" s="29" t="s">
         <v>27</v>
@@ -1234,7 +1273,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" s="29" t="s">
         <v>27</v>
@@ -1248,7 +1287,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="29" t="s">
         <v>27</v>
@@ -1259,7 +1298,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C9" s="34" t="s">
         <v>1</v>
@@ -1304,7 +1343,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" s="29" t="s">
         <v>45</v>
@@ -1318,15 +1357,15 @@
         <v>32</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="0"/>
       <c r="D14" s="0"/>
@@ -1353,120 +1392,120 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="59" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="58" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="58" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="58" t="s">
+      <c r="A1" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="16" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="57" t="s">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="54" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="55" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="56" t="s">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="51" t="s">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="46" t="s">
+      <c r="C4" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="20" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="53" t="s">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="49" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" s="50" t="s">
+      <c r="C5" s="42" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="43" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="51" t="s">
+      <c r="A6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="45" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6" s="46" t="s">
+      <c r="C6" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="53" t="s">
+      <c r="A7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="50" t="s">
+      <c r="C7" s="42" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="43" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="52" t="s">
+      <c r="A8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="48" t="s">
-        <v>24</v>
+      <c r="C8" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="41" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0"/>
@@ -1478,4 +1517,230 @@
     <mergeCell ref="B9:D9"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
+    <col min="2" max="2" width="17.7109375" style="1" customWidth="true"/>
+    <col min="3" max="3" width="8.7109375" style="1" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="1" customWidth="true"/>
+    <col min="5" max="5" width="8.7109375" style="1" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C2:E2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
+    <col min="2" max="2" width="17.7109375" style="1" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" style="1" customWidth="true"/>
+    <col min="4" max="4" width="18.7109375" style="1" customWidth="true"/>
+    <col min="5" max="5" width="16.7109375" style="1" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="55" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="55" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="55" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="55" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="54" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="53" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="51" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>